<commit_message>
New Estimations and Files
</commit_message>
<xml_diff>
--- a/R/Input/DATAc.xlsx
+++ b/R/Input/DATAc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bancodelarepublica-my.sharepoint.com/personal/ojaulime_banrep_gov_co/Documents/Documents/Research/MP transmission in Colombia/Monetary-Policy-Shocks-and-Central-bank-information-in-Colombia/R/Input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Disco C\Repositorios Git\Monetary-Policy-Shocks-and-Central-bank-information-in-Colombia\R\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{61A7BA06-15EE-486E-B896-9040FC5EED2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E261624B-1EA4-406E-877D-E4527EBB6D47}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{5935AB3E-80CE-4E87-9EB4-B18D2E64BDED}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{5935AB3E-80CE-4E87-9EB4-B18D2E64BDED}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -83,8 +83,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -133,13 +133,13 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -156,10 +156,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -460,9 +456,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11DADDA8-F05A-4B81-9CDB-818A1AD50DCA}">
   <dimension ref="A1:N253"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -506,7 +502,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>38353</v>
       </c>
@@ -529,7 +525,7 @@
         <v>4.5591700000000004E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>38384</v>
       </c>
@@ -552,7 +548,7 @@
         <v>1.36775E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>38412</v>
       </c>
@@ -575,7 +571,7 @@
         <v>0.11486080999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>38443</v>
       </c>
@@ -598,7 +594,7 @@
         <v>5.4710000000000002E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>38473</v>
       </c>
@@ -621,7 +617,7 @@
         <v>2.2645E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>38504</v>
       </c>
@@ -644,7 +640,7 @@
         <v>-5.5011599999999997E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>38534</v>
       </c>
@@ -667,7 +663,7 @@
         <v>-2.826683E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>38565</v>
       </c>
@@ -690,7 +686,7 @@
         <v>4.5592000000000001E-4</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>38596</v>
       </c>
@@ -713,7 +709,7 @@
         <v>-0.23819141999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>38626</v>
       </c>
@@ -736,7 +732,7 @@
         <v>2.860209E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>38657</v>
       </c>
@@ -759,7 +755,7 @@
         <v>-1.8236699999999999E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>38687</v>
       </c>
@@ -782,7 +778,7 @@
         <v>3.1914159999999997E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>38718</v>
       </c>
@@ -805,7 +801,7 @@
         <v>3.1914199999999999E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>38749</v>
       </c>
@@ -828,7 +824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>38777</v>
       </c>
@@ -851,7 +847,7 @@
         <v>5.9269199999999996E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>38808</v>
       </c>
@@ -874,7 +870,7 @@
         <v>7.2976819999999998E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>38838</v>
       </c>
@@ -897,7 +893,7 @@
         <v>-0.11150349</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>38869</v>
       </c>
@@ -920,7 +916,7 @@
         <v>1.5440829999999999E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>38899</v>
       </c>
@@ -943,7 +939,7 @@
         <v>-9.8828319999999997E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>38930</v>
       </c>
@@ -966,7 +962,7 @@
         <v>8.6171700000000004E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>38961</v>
       </c>
@@ -989,7 +985,7 @@
         <v>7.2720419999999994E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>38991</v>
       </c>
@@ -1012,7 +1008,7 @@
         <v>5.8236660000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>39022</v>
       </c>
@@ -1035,7 +1031,7 @@
         <v>-2.591183E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>39052</v>
       </c>
@@ -1058,7 +1054,7 @@
         <v>0.10091182999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>39083</v>
       </c>
@@ -1081,7 +1077,7 @@
         <v>2.305567E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>39114</v>
       </c>
@@ -1104,7 +1100,7 @@
         <v>-0.11212531000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>39142</v>
       </c>
@@ -1127,7 +1123,7 @@
         <v>-3.2370080000000002E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>39173</v>
       </c>
@@ -1150,7 +1146,7 @@
         <v>-4.529E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>39203</v>
       </c>
@@ -1173,7 +1169,7 @@
         <v>-0.23709169999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>39234</v>
       </c>
@@ -1196,7 +1192,7 @@
         <v>-5.8933899999999997E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>39264</v>
       </c>
@@ -1219,7 +1215,7 @@
         <v>5.5911830000000003E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>39295</v>
       </c>
@@ -1242,7 +1238,7 @@
         <v>-5.674825E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>39326</v>
       </c>
@@ -1265,7 +1261,7 @@
         <v>-0.23797336999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>39356</v>
       </c>
@@ -1288,7 +1284,7 @@
         <v>-0.25985736999999998</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>39387</v>
       </c>
@@ -1311,7 +1307,7 @@
         <v>0.11908816999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>39417</v>
       </c>
@@ -1334,7 +1330,7 @@
         <v>0.23253254000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>39448</v>
       </c>
@@ -1378,7 +1374,7 @@
         <v>-4.2562299999999997E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>39479</v>
       </c>
@@ -1422,7 +1418,7 @@
         <v>5.9226639999999997E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>39508</v>
       </c>
@@ -1466,7 +1462,7 @@
         <v>0.32610652000000001</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>39539</v>
       </c>
@@ -1510,7 +1506,7 @@
         <v>0.36944381999999998</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>39569</v>
       </c>
@@ -1554,7 +1550,7 @@
         <v>-0.44944381999999999</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>39600</v>
       </c>
@@ -1598,7 +1594,7 @@
         <v>-0.44350611000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
         <v>39630</v>
       </c>
@@ -1642,7 +1638,7 @@
         <v>0.46301308000000002</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>39661</v>
       </c>
@@ -1686,7 +1682,7 @@
         <v>-4.4953279999999998E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
         <v>39692</v>
       </c>
@@ -1730,7 +1726,7 @@
         <v>-6.0536899999999996E-3</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>39722</v>
       </c>
@@ -1774,7 +1770,7 @@
         <v>-0.49770323999999999</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
         <v>39753</v>
       </c>
@@ -1818,7 +1814,7 @@
         <v>-0.38327783999999998</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
         <v>39783</v>
       </c>
@@ -1862,7 +1858,7 @@
         <v>0.15606513999999999</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" s="1">
         <v>39814</v>
       </c>
@@ -1906,7 +1902,7 @@
         <v>-0.47338358000000003</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" s="1">
         <v>39845</v>
       </c>
@@ -1950,7 +1946,7 @@
         <v>-0.54739097999999997</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" s="1">
         <v>39873</v>
       </c>
@@ -1994,7 +1990,7 @@
         <v>-0.51314877000000003</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" s="1">
         <v>39904</v>
       </c>
@@ -2038,7 +2034,7 @@
         <v>-0.55107950000000006</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" s="1">
         <v>39934</v>
       </c>
@@ -2082,7 +2078,7 @@
         <v>-0.50324221000000002</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" s="1">
         <v>39965</v>
       </c>
@@ -2126,7 +2122,7 @@
         <v>-0.63880201999999997</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" s="1">
         <v>39995</v>
       </c>
@@ -2170,7 +2166,7 @@
         <v>1.3102050000000001E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" s="1">
         <v>40026</v>
       </c>
@@ -2214,7 +2210,7 @@
         <v>6.4171309999999995E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" s="1">
         <v>40057</v>
       </c>
@@ -2258,7 +2254,7 @@
         <v>-0.24067295</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" s="1">
         <v>40087</v>
       </c>
@@ -2302,7 +2298,7 @@
         <v>-1.2484429999999999E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" s="1">
         <v>40118</v>
       </c>
@@ -2346,7 +2342,7 @@
         <v>-0.35513646999999998</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" s="1">
         <v>40148</v>
       </c>
@@ -2390,7 +2386,7 @@
         <v>0.12279754</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" s="1">
         <v>40179</v>
       </c>
@@ -2434,7 +2430,7 @@
         <v>0.11314877</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" s="1">
         <v>40210</v>
       </c>
@@ -2478,7 +2474,7 @@
         <v>0.10201721</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="1">
         <v>40238</v>
       </c>
@@ -2522,7 +2518,7 @@
         <v>3.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" s="1">
         <v>40269</v>
       </c>
@@ -2566,7 +2562,7 @@
         <v>-0.27829754000000001</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" s="1">
         <v>40299</v>
       </c>
@@ -2610,7 +2606,7 @@
         <v>-3.0679919999999999E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" s="1">
         <v>40330</v>
       </c>
@@ -2654,7 +2650,7 @@
         <v>-3.0679919999999999E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" s="1">
         <v>40360</v>
       </c>
@@ -2698,7 +2694,7 @@
         <v>-3.2695490000000001E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69" s="1">
         <v>40391</v>
       </c>
@@ -2742,7 +2738,7 @@
         <v>0.19299957000000001</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70" s="1">
         <v>40422</v>
       </c>
@@ -2786,7 +2782,7 @@
         <v>-0.15866063999999999</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71" s="1">
         <v>40452</v>
       </c>
@@ -2830,7 +2826,7 @@
         <v>-2.303115E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" s="1">
         <v>40483</v>
       </c>
@@ -2874,7 +2870,7 @@
         <v>0.11330941</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73" s="1">
         <v>40513</v>
       </c>
@@ -2918,7 +2914,7 @@
         <v>-4.4633199999999998E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74" s="1">
         <v>40544</v>
       </c>
@@ -2962,7 +2958,7 @@
         <v>-2.235123E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75" s="1">
         <v>40575</v>
       </c>
@@ -3006,7 +3002,7 @@
         <v>9.36332E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76" s="1">
         <v>40603</v>
       </c>
@@ -3050,7 +3046,7 @@
         <v>0.24520900000000001</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77" s="1">
         <v>40634</v>
       </c>
@@ -3094,7 +3090,7 @@
         <v>2.351557E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A78" s="1">
         <v>40664</v>
       </c>
@@ -3138,7 +3134,7 @@
         <v>5.9281970000000003E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A79" s="1">
         <v>40695</v>
       </c>
@@ -3182,7 +3178,7 @@
         <v>6.0484429999999999E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A80" s="1">
         <v>40725</v>
       </c>
@@ -3226,7 +3222,7 @@
         <v>2.2031149999999999E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A81" s="1">
         <v>40756</v>
       </c>
@@ -3270,7 +3266,7 @@
         <v>-0.23957581</v>
       </c>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A82" s="1">
         <v>40787</v>
       </c>
@@ -3314,7 +3310,7 @@
         <v>-4.789098E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A83" s="1">
         <v>40817</v>
       </c>
@@ -3358,7 +3354,7 @@
         <v>-5.9437700000000003E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A84" s="1">
         <v>40848</v>
       </c>
@@ -3402,7 +3398,7 @@
         <v>4.510902E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A85" s="1">
         <v>40878</v>
       </c>
@@ -3446,7 +3442,7 @@
         <v>-3.4757789999999997E-2</v>
       </c>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A86" s="1">
         <v>40909</v>
       </c>
@@ -3490,7 +3486,7 @@
         <v>0.11464877</v>
       </c>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A87" s="1">
         <v>40940</v>
       </c>
@@ -3534,7 +3530,7 @@
         <v>8.6711070000000001E-2</v>
       </c>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A88" s="1">
         <v>40969</v>
       </c>
@@ -3578,7 +3574,7 @@
         <v>-1.2164339999999999E-2</v>
       </c>
     </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A89" s="1">
         <v>41000</v>
       </c>
@@ -3622,7 +3618,7 @@
         <v>-1.2437699999999999E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A90" s="1">
         <v>41030</v>
       </c>
@@ -3666,7 +3662,7 @@
         <v>-0.23711719000000001</v>
       </c>
     </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A91" s="1">
         <v>41061</v>
       </c>
@@ -3710,7 +3706,7 @@
         <v>-2.275779E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A92" s="1">
         <v>41091</v>
       </c>
@@ -3754,7 +3750,7 @@
         <v>-0.18792212999999999</v>
       </c>
     </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A93" s="1">
         <v>41122</v>
       </c>
@@ -3798,7 +3794,7 @@
         <v>-4.3515570000000003E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A94" s="1">
         <v>41153</v>
       </c>
@@ -3842,7 +3838,7 @@
         <v>-8.2380309999999998E-2</v>
       </c>
     </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A95" s="1">
         <v>41183</v>
       </c>
@@ -3886,7 +3882,7 @@
         <v>1.7195490000000001E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A96" s="1">
         <v>41214</v>
       </c>
@@ -3930,7 +3926,7 @@
         <v>-0.22312088999999999</v>
       </c>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A97" s="1">
         <v>41244</v>
       </c>
@@ -3974,7 +3970,7 @@
         <v>-3.877336E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A98" s="1">
         <v>41275</v>
       </c>
@@ -4018,7 +4014,7 @@
         <v>1.8468849999999998E-2</v>
       </c>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A99" s="1">
         <v>41306</v>
       </c>
@@ -4062,7 +4058,7 @@
         <v>0.12164506999999999</v>
       </c>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A100" s="1">
         <v>41334</v>
       </c>
@@ -4106,7 +4102,7 @@
         <v>-0.24754302</v>
       </c>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A101" s="1">
         <v>41365</v>
       </c>
@@ -4150,7 +4146,7 @@
         <v>0.17684753</v>
       </c>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A102" s="1">
         <v>41395</v>
       </c>
@@ -4194,7 +4190,7 @@
         <v>0.16510695</v>
       </c>
     </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A103" s="1">
         <v>41426</v>
       </c>
@@ -4238,7 +4234,7 @@
         <v>0.20424875000000001</v>
       </c>
     </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A104" s="1">
         <v>41456</v>
       </c>
@@ -4282,7 +4278,7 @@
         <v>0.14866925</v>
       </c>
     </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A105" s="1">
         <v>41487</v>
       </c>
@@ -4326,7 +4322,7 @@
         <v>-0.14827826999999999</v>
       </c>
     </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A106" s="1">
         <v>41518</v>
       </c>
@@ -4370,7 +4366,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A107" s="1">
         <v>41548</v>
       </c>
@@ -4414,7 +4410,7 @@
         <v>1.72664E-3</v>
       </c>
     </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A108" s="1">
         <v>41579</v>
       </c>
@@ -4458,7 +4454,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A109" s="1">
         <v>41609</v>
       </c>
@@ -4502,7 +4498,7 @@
         <v>9.9688499999999996E-3</v>
       </c>
     </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A110" s="1">
         <v>41640</v>
       </c>
@@ -4546,7 +4542,7 @@
         <v>-5.3045100000000001E-3</v>
       </c>
     </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A111" s="1">
         <v>41671</v>
       </c>
@@ -4590,7 +4586,7 @@
         <v>-3.9844299999999997E-3</v>
       </c>
     </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A112" s="1">
         <v>41699</v>
       </c>
@@ -4634,7 +4630,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A113" s="1">
         <v>41730</v>
       </c>
@@ -4678,7 +4674,7 @@
         <v>0.12378893000000001</v>
       </c>
     </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A114" s="1">
         <v>41760</v>
       </c>
@@ -4722,7 +4718,7 @@
         <v>2.0359829999999999E-2</v>
       </c>
     </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A115" s="1">
         <v>41791</v>
       </c>
@@ -4766,7 +4762,7 @@
         <v>-2.44377E-2</v>
       </c>
     </row>
-    <row r="116" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A116" s="1">
         <v>41821</v>
       </c>
@@ -4810,7 +4806,7 @@
         <v>6.5617620000000002E-2</v>
       </c>
     </row>
-    <row r="117" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A117" s="1">
         <v>41852</v>
       </c>
@@ -4854,7 +4850,7 @@
         <v>5.6788930000000001E-2</v>
       </c>
     </row>
-    <row r="118" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A118" s="1">
         <v>41883</v>
       </c>
@@ -4898,7 +4894,7 @@
         <v>9.1799199999999994E-3</v>
       </c>
     </row>
-    <row r="119" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A119" s="1">
         <v>41913</v>
       </c>
@@ -4942,7 +4938,7 @@
         <v>-2.3993029999999999E-2</v>
       </c>
     </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A120" s="1">
         <v>41944</v>
       </c>
@@ -4986,7 +4982,7 @@
         <v>5.1557000000000003E-4</v>
       </c>
     </row>
-    <row r="121" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A121" s="1">
         <v>41974</v>
       </c>
@@ -5030,7 +5026,7 @@
         <v>-5.0954909999999999E-2</v>
       </c>
     </row>
-    <row r="122" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A122" s="1">
         <v>42005</v>
       </c>
@@ -5074,7 +5070,7 @@
         <v>2.9688499999999999E-3</v>
       </c>
     </row>
-    <row r="123" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A123" s="1">
         <v>42036</v>
       </c>
@@ -5118,7 +5114,7 @@
         <v>2.5778999999999998E-4</v>
       </c>
     </row>
-    <row r="124" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A124" s="1">
         <v>42064</v>
       </c>
@@ -5162,7 +5158,7 @@
         <v>-4.95328E-3</v>
       </c>
     </row>
-    <row r="125" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A125" s="1">
         <v>42095</v>
       </c>
@@ -5206,7 +5202,7 @@
         <v>1.403975E-2</v>
       </c>
     </row>
-    <row r="126" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A126" s="1">
         <v>42125</v>
       </c>
@@ -5250,7 +5246,7 @@
         <v>-2.181311E-2</v>
       </c>
     </row>
-    <row r="127" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A127" s="1">
         <v>42156</v>
       </c>
@@ -5294,7 +5290,7 @@
         <v>-1.069549E-2</v>
       </c>
     </row>
-    <row r="128" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A128" s="1">
         <v>42186</v>
       </c>
@@ -5338,7 +5334,7 @@
         <v>7.4930300000000003E-3</v>
       </c>
     </row>
-    <row r="129" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A129" s="1">
         <v>42217</v>
       </c>
@@ -5382,7 +5378,7 @@
         <v>-5.9726639999999998E-2</v>
       </c>
     </row>
-    <row r="130" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A130" s="1">
         <v>42248</v>
       </c>
@@ -5426,7 +5422,7 @@
         <v>7.5437699999999996E-2</v>
       </c>
     </row>
-    <row r="131" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A131" s="1">
         <v>42278</v>
       </c>
@@ -5470,7 +5466,7 @@
         <v>8.803975E-2</v>
       </c>
     </row>
-    <row r="132" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A132" s="1">
         <v>42309</v>
       </c>
@@ -5514,7 +5510,7 @@
         <v>-7.4226639999999997E-2</v>
       </c>
     </row>
-    <row r="133" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A133" s="1">
         <v>42339</v>
       </c>
@@ -5558,7 +5554,7 @@
         <v>-3.927336E-2</v>
       </c>
     </row>
-    <row r="134" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A134" s="1">
         <v>42370</v>
       </c>
@@ -5602,7 +5598,7 @@
         <v>-4.3242210000000003E-2</v>
       </c>
     </row>
-    <row r="135" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A135" s="1">
         <v>42401</v>
       </c>
@@ -5646,7 +5642,7 @@
         <v>-4.5211069999999999E-2</v>
       </c>
     </row>
-    <row r="136" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A136" s="1">
         <v>42430</v>
       </c>
@@ -5690,7 +5686,7 @@
         <v>2.9679919999999999E-2</v>
       </c>
     </row>
-    <row r="137" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A137" s="1">
         <v>42461</v>
       </c>
@@ -5734,7 +5730,7 @@
         <v>0.10966434</v>
       </c>
     </row>
-    <row r="138" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A138" s="1">
         <v>42491</v>
       </c>
@@ -5778,7 +5774,7 @@
         <v>-1.8288929999999998E-2</v>
       </c>
     </row>
-    <row r="139" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A139" s="1">
         <v>42522</v>
       </c>
@@ -5822,7 +5818,7 @@
         <v>-5.4844300000000002E-3</v>
       </c>
     </row>
-    <row r="140" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A140" s="1">
         <v>42552</v>
       </c>
@@ -5866,7 +5862,7 @@
         <v>-6.5172099999999998E-3</v>
       </c>
     </row>
-    <row r="141" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A141" s="1">
         <v>42583</v>
       </c>
@@ -5910,7 +5906,7 @@
         <v>-5.7133200000000002E-2</v>
       </c>
     </row>
-    <row r="142" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A142" s="1">
         <v>42614</v>
       </c>
@@ -5954,7 +5950,7 @@
         <v>-2.4688499999999999E-3</v>
       </c>
     </row>
-    <row r="143" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A143" s="1">
         <v>42644</v>
       </c>
@@ -5998,7 +5994,7 @@
         <v>1.5155699999999999E-3</v>
       </c>
     </row>
-    <row r="144" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A144" s="1">
         <v>42675</v>
       </c>
@@ -6042,7 +6038,7 @@
         <v>4.7110700000000004E-3</v>
       </c>
     </row>
-    <row r="145" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A145" s="1">
         <v>42705</v>
       </c>
@@ -6086,7 +6082,7 @@
         <v>-0.10871107000000001</v>
       </c>
     </row>
-    <row r="146" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A146" s="1">
         <v>42736</v>
       </c>
@@ -6130,7 +6126,7 @@
         <v>9.5875409999999994E-2</v>
       </c>
     </row>
-    <row r="147" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A147" s="1">
         <v>42767</v>
       </c>
@@ -6174,7 +6170,7 @@
         <v>-7.9695489999999994E-2</v>
       </c>
     </row>
-    <row r="148" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A148" s="1">
         <v>42795</v>
       </c>
@@ -6218,7 +6214,7 @@
         <v>4.9257790000000003E-2</v>
       </c>
     </row>
-    <row r="149" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A149" s="1">
         <v>42826</v>
       </c>
@@ -6262,7 +6258,7 @@
         <v>-2.814877E-2</v>
       </c>
     </row>
-    <row r="150" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A150" s="1">
         <v>42856</v>
       </c>
@@ -6306,7 +6302,7 @@
         <v>4.8757790000000002E-2</v>
       </c>
     </row>
-    <row r="151" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A151" s="1">
         <v>42887</v>
       </c>
@@ -6350,7 +6346,7 @@
         <v>-2.2313110000000001E-2</v>
       </c>
     </row>
-    <row r="152" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A152" s="1">
         <v>42917</v>
       </c>
@@ -6394,7 +6390,7 @@
         <v>3.5015570000000003E-2</v>
       </c>
     </row>
-    <row r="153" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A153" s="1">
         <v>42948</v>
       </c>
@@ -6438,7 +6434,7 @@
         <v>1.6726640000000001E-2</v>
       </c>
     </row>
-    <row r="154" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A154" s="1">
         <v>42979</v>
       </c>
@@ -6482,7 +6478,7 @@
         <v>3.7211069999999999E-2</v>
       </c>
     </row>
-    <row r="155" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A155" s="1">
         <v>43009</v>
       </c>
@@ -6526,7 +6522,7 @@
         <v>-0.10117992000000001</v>
       </c>
     </row>
-    <row r="156" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A156" s="1">
         <v>43040</v>
       </c>
@@ -6570,7 +6566,7 @@
         <v>-3.2179920000000001E-2</v>
       </c>
     </row>
-    <row r="157" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A157" s="1">
         <v>43070</v>
       </c>
@@ -6614,7 +6610,7 @@
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="158" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A158" s="1">
         <v>43101</v>
       </c>
@@ -6658,7 +6654,7 @@
         <v>-6.0288929999999998E-2</v>
       </c>
     </row>
-    <row r="159" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A159" s="1">
         <v>43132</v>
       </c>
@@ -6702,7 +6698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A160" s="1">
         <v>43160</v>
       </c>
@@ -6746,7 +6742,7 @@
         <v>3.2515570000000001E-2</v>
       </c>
     </row>
-    <row r="161" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A161" s="1">
         <v>43191</v>
       </c>
@@ -6790,7 +6786,7 @@
         <v>1.4532799999999999E-3</v>
       </c>
     </row>
-    <row r="162" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A162" s="1">
         <v>43221</v>
       </c>
@@ -6834,7 +6830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A163" s="1">
         <v>43252</v>
       </c>
@@ -6878,7 +6874,7 @@
         <v>-1.808647E-2</v>
       </c>
     </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A164" s="1">
         <v>43282</v>
       </c>
@@ -6922,7 +6918,7 @@
         <v>-2.152418E-2</v>
       </c>
     </row>
-    <row r="165" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A165" s="1">
         <v>43313</v>
       </c>
@@ -6966,7 +6962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A166" s="1">
         <v>43344</v>
       </c>
@@ -7010,7 +7006,7 @@
         <v>5.0000000000000001E-4</v>
       </c>
     </row>
-    <row r="167" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A167" s="1">
         <v>43374</v>
       </c>
@@ -7054,7 +7050,7 @@
         <v>-1E-3</v>
       </c>
     </row>
-    <row r="168" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A168" s="1">
         <v>43405</v>
       </c>
@@ -7098,7 +7094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A169" s="1">
         <v>43435</v>
       </c>
@@ -7142,7 +7138,7 @@
         <v>5.9377039999999999E-2</v>
       </c>
     </row>
-    <row r="170" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A170" s="1">
         <v>43466</v>
       </c>
@@ -7186,7 +7182,7 @@
         <v>1.0390979999999999E-2</v>
       </c>
     </row>
-    <row r="171" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A171" s="1">
         <v>43497</v>
       </c>
@@ -7230,7 +7226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A172" s="1">
         <v>43525</v>
       </c>
@@ -7274,7 +7270,7 @@
         <v>-6.1799200000000002E-3</v>
       </c>
     </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A173" s="1">
         <v>43556</v>
       </c>
@@ -7318,7 +7314,7 @@
         <v>9.6487699999999992E-3</v>
       </c>
     </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A174" s="1">
         <v>43586</v>
       </c>
@@ -7362,7 +7358,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A175" s="1">
         <v>43617</v>
       </c>
@@ -7406,7 +7402,7 @@
         <v>8.6799200000000007E-3</v>
       </c>
     </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A176" s="1">
         <v>43647</v>
       </c>
@@ -7450,7 +7446,7 @@
         <v>5.4999999999999997E-3</v>
       </c>
     </row>
-    <row r="177" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A177" s="1">
         <v>43678</v>
       </c>
@@ -7494,7 +7490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A178" s="1">
         <v>43709</v>
       </c>
@@ -7538,7 +7534,7 @@
         <v>2.4221E-4</v>
       </c>
     </row>
-    <row r="179" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A179" s="1">
         <v>43739</v>
       </c>
@@ -7582,7 +7578,7 @@
         <v>9.2761060000000006E-2</v>
       </c>
     </row>
-    <row r="180" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A180" s="1">
         <v>43770</v>
       </c>
@@ -7626,7 +7622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A181" s="1">
         <v>43800</v>
       </c>
@@ -7670,7 +7666,7 @@
         <v>7.6447940000000006E-2</v>
       </c>
     </row>
-    <row r="182" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="182" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A182" s="1">
         <v>43831</v>
       </c>
@@ -7714,7 +7710,7 @@
         <v>-1.5602049999999999E-2</v>
       </c>
     </row>
-    <row r="183" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="183" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A183" s="1">
         <v>43862</v>
       </c>
@@ -7758,7 +7754,7 @@
         <v>-5.0000000000000001E-4</v>
       </c>
     </row>
-    <row r="184" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="184" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A184" s="1">
         <v>43891</v>
       </c>
@@ -7802,7 +7798,7 @@
         <v>-4.630451E-2</v>
       </c>
     </row>
-    <row r="185" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="185" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A185" s="1">
         <v>43922</v>
       </c>
@@ -7846,7 +7842,7 @@
         <v>4.814877E-2</v>
       </c>
     </row>
-    <row r="186" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="186" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A186" s="1">
         <v>43952</v>
       </c>
@@ -7890,7 +7886,7 @@
         <v>-9.6331999999999997E-3</v>
       </c>
     </row>
-    <row r="187" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="187" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A187" s="1">
         <v>43983</v>
       </c>
@@ -7934,7 +7930,7 @@
         <v>8.1890980000000002E-2</v>
       </c>
     </row>
-    <row r="188" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="188" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A188" s="1">
         <v>44013</v>
       </c>
@@ -7978,7 +7974,7 @@
         <v>6.6176200000000003E-3</v>
       </c>
     </row>
-    <row r="189" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="189" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A189" s="1">
         <v>44044</v>
       </c>
@@ -8022,7 +8018,7 @@
         <v>-1.6077870000000001E-2</v>
       </c>
     </row>
-    <row r="190" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="190" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A190" s="1">
         <v>44075</v>
       </c>
@@ -8066,7 +8062,7 @@
         <v>-7.4890979999999996E-2</v>
       </c>
     </row>
-    <row r="191" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="191" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A191" s="1">
         <v>44105</v>
       </c>
@@ -8110,7 +8106,7 @@
         <v>-7.2663999999999997E-4</v>
       </c>
     </row>
-    <row r="192" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="192" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A192" s="1">
         <v>44136</v>
       </c>
@@ -8154,7 +8150,7 @@
         <v>-3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="193" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="193" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A193" s="1">
         <v>44166</v>
       </c>
@@ -8198,7 +8194,7 @@
         <v>8.1487699999999996E-3</v>
       </c>
     </row>
-    <row r="194" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="194" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A194" s="1">
         <v>44197</v>
       </c>
@@ -8242,7 +8238,7 @@
         <v>1.424221E-2</v>
       </c>
     </row>
-    <row r="195" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="195" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A195" s="1">
         <v>44228</v>
       </c>
@@ -8286,7 +8282,7 @@
         <v>-5.0000000000000001E-4</v>
       </c>
     </row>
-    <row r="196" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="196" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A196" s="1">
         <v>44256</v>
       </c>
@@ -8330,7 +8326,7 @@
         <v>1.2390979999999999E-2</v>
       </c>
     </row>
-    <row r="197" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="197" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A197" s="1">
         <v>44287</v>
       </c>
@@ -8374,7 +8370,7 @@
         <v>1.5375410000000001E-2</v>
       </c>
     </row>
-    <row r="198" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="198" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A198" s="1">
         <v>44317</v>
       </c>
@@ -8418,7 +8414,7 @@
         <v>-3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="199" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="199" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A199" s="1">
         <v>44348</v>
       </c>
@@ -8462,7 +8458,7 @@
         <v>-1.0320080000000001E-2</v>
       </c>
     </row>
-    <row r="200" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="200" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A200" s="1">
         <v>44378</v>
       </c>
@@ -8506,7 +8502,7 @@
         <v>1.72664E-3</v>
       </c>
     </row>
-    <row r="201" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="201" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A201" s="1">
         <v>44409</v>
       </c>
@@ -8550,7 +8546,7 @@
         <v>-1.15E-2</v>
       </c>
     </row>
-    <row r="202" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="202" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A202" s="1">
         <v>44440</v>
       </c>
@@ -8594,7 +8590,7 @@
         <v>-3.853115E-2</v>
       </c>
     </row>
-    <row r="203" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="203" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A203" s="1">
         <v>44470</v>
       </c>
@@ -8638,7 +8634,7 @@
         <v>4.9875410000000002E-2</v>
       </c>
     </row>
-    <row r="204" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="204" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A204" s="1">
         <v>44501</v>
       </c>
@@ -8682,7 +8678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="205" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A205" s="1">
         <v>44531</v>
       </c>
@@ -8726,7 +8722,7 @@
         <v>-5.7820080000000003E-2</v>
       </c>
     </row>
-    <row r="206" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="206" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A206" s="1">
         <v>44562</v>
       </c>
@@ -8770,7 +8766,7 @@
         <v>7.2437699999999994E-2</v>
       </c>
     </row>
-    <row r="207" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="207" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A207" s="1">
         <v>44593</v>
       </c>
@@ -8814,7 +8810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="208" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A208" s="1">
         <v>44621</v>
       </c>
@@ -8858,7 +8854,7 @@
         <v>-0.25576639000000001</v>
       </c>
     </row>
-    <row r="209" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="209" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A209" s="1">
         <v>44652</v>
       </c>
@@ -8902,7 +8898,7 @@
         <v>-8.1557399999999999E-3</v>
       </c>
     </row>
-    <row r="210" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="210" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A210" s="1">
         <v>44682</v>
       </c>
@@ -8946,7 +8942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:14" ht="15.5" x14ac:dyDescent="0.4">
+    <row r="211" spans="1:14" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A211" s="1">
         <v>44713</v>
       </c>
@@ -8990,7 +8986,7 @@
         <v>2.2422100000000001E-3</v>
       </c>
     </row>
-    <row r="212" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A212" s="1">
         <v>44743</v>
       </c>
@@ -9034,7 +9030,7 @@
         <v>4.0467200000000002E-3</v>
       </c>
     </row>
-    <row r="213" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A213" s="1">
         <v>44774</v>
       </c>
@@ -9078,7 +9074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A214" s="1">
         <v>44805</v>
       </c>
@@ -9122,7 +9118,7 @@
         <v>-0.18711762000000001</v>
       </c>
     </row>
-    <row r="215" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A215" s="1">
         <v>44835</v>
       </c>
@@ -9166,7 +9162,7 @@
         <v>1.6487699999999999E-3</v>
       </c>
     </row>
-    <row r="216" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A216" s="1">
         <v>44866</v>
       </c>
@@ -9210,7 +9206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A217" s="1">
         <v>44896</v>
       </c>
@@ -9254,7 +9250,7 @@
         <v>0.10050000000000001</v>
       </c>
     </row>
-    <row r="218" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A218" s="1">
         <v>44927</v>
       </c>
@@ -9298,7 +9294,7 @@
         <v>5.1148770000000003E-2</v>
       </c>
     </row>
-    <row r="219" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A219" s="1">
         <v>44958</v>
       </c>
@@ -9342,7 +9338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A220" s="1">
         <v>44986</v>
       </c>
@@ -9386,7 +9382,7 @@
         <v>1.30451E-3</v>
       </c>
     </row>
-    <row r="221" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A221" s="1">
         <v>45017</v>
       </c>
@@ -9430,7 +9426,7 @@
         <v>7.8375410000000006E-2</v>
       </c>
     </row>
-    <row r="222" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A222" s="1">
         <v>45047</v>
       </c>
@@ -9474,7 +9470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A223" s="1">
         <v>45078</v>
       </c>
@@ -9518,7 +9514,7 @@
         <v>1.287541E-2</v>
       </c>
     </row>
-    <row r="224" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A224" s="1">
         <v>45108</v>
       </c>
@@ -9562,7 +9558,7 @@
         <v>5.1954899999999997E-3</v>
       </c>
     </row>
-    <row r="225" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A225" s="1">
         <v>45139</v>
       </c>
@@ -9606,7 +9602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A226" s="1">
         <v>45170</v>
       </c>
@@ -9650,7 +9646,7 @@
         <v>1.069549E-2</v>
       </c>
     </row>
-    <row r="227" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A227" s="1">
         <v>45200</v>
       </c>
@@ -9694,7 +9690,7 @@
         <v>6.1799200000000002E-3</v>
       </c>
     </row>
-    <row r="228" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A228" s="1">
         <v>45231</v>
       </c>
@@ -9738,7 +9734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A229" s="1">
         <v>45261</v>
       </c>
@@ -9782,7 +9778,7 @@
         <v>-4.7773360000000001E-2</v>
       </c>
     </row>
-    <row r="230" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A230" s="1">
         <v>45292</v>
       </c>
@@ -9826,7 +9822,7 @@
         <v>8.7046719999999994E-2</v>
       </c>
     </row>
-    <row r="231" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A231" s="1">
         <v>45323</v>
       </c>
@@ -9870,7 +9866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A232" s="1">
         <v>45352</v>
       </c>
@@ -9914,7 +9910,7 @@
         <v>-3.0623E-3</v>
       </c>
     </row>
-    <row r="233" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A233" s="1">
         <v>45383</v>
       </c>
@@ -9958,7 +9954,7 @@
         <v>-1.322664E-2</v>
       </c>
     </row>
-    <row r="234" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A234" s="1">
         <v>45413</v>
       </c>
@@ -10002,7 +9998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A235" s="1">
         <v>45444</v>
       </c>
@@ -10046,7 +10042,7 @@
         <v>-7.729221E-2</v>
       </c>
     </row>
-    <row r="236" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A236" s="1">
         <v>45474</v>
       </c>
@@ -10090,7 +10086,7 @@
         <v>5.25779E-3</v>
       </c>
     </row>
-    <row r="237" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A237" s="1">
         <v>45505</v>
       </c>
@@ -10134,7 +10130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A238" s="1">
         <v>45536</v>
       </c>
@@ -10178,7 +10174,7 @@
         <v>3.974221E-2</v>
       </c>
     </row>
-    <row r="239" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A239" s="1">
         <v>45566</v>
       </c>
@@ -10222,7 +10218,7 @@
         <v>2.111762E-2</v>
       </c>
     </row>
-    <row r="240" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A240" s="1">
         <v>45597</v>
       </c>
@@ -10266,7 +10262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A241" s="1">
         <v>45627</v>
       </c>
@@ -10310,7 +10306,7 @@
         <v>0.19940121999999999</v>
       </c>
     </row>
-    <row r="242" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A242" s="1">
         <v>45658</v>
       </c>
@@ -10354,7 +10350,7 @@
         <v>7.1757790000000002E-2</v>
       </c>
     </row>
-    <row r="243" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A243" s="1">
         <v>45689</v>
       </c>
@@ -10398,7 +10394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A244" s="1">
         <v>45717</v>
       </c>
@@ -10442,7 +10438,7 @@
         <v>-7.4220999999999998E-4</v>
       </c>
     </row>
-    <row r="245" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A245" s="1">
         <v>45748</v>
       </c>
@@ -10486,7 +10482,7 @@
         <v>-9.5311480000000004E-2</v>
       </c>
     </row>
-    <row r="246" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A246" s="1">
         <v>45778</v>
       </c>
@@ -10530,7 +10526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A247" s="1">
         <v>45809</v>
       </c>
@@ -10574,7 +10570,7 @@
         <v>-7.4221299999999999E-3</v>
       </c>
     </row>
-    <row r="248" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A248" s="1">
         <v>45839</v>
       </c>
@@ -10588,7 +10584,7 @@
         <v>9.2469565217391317E-2</v>
       </c>
     </row>
-    <row r="249" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A249" s="1">
         <v>45870</v>
       </c>
@@ -10602,7 +10598,7 @@
         <v>9.2478947368421063E-2</v>
       </c>
     </row>
-    <row r="250" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A250" s="1">
         <v>45901</v>
       </c>
@@ -10616,7 +10612,7 @@
         <v>9.2481818181818193E-2</v>
       </c>
     </row>
-    <row r="251" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A251" s="1">
         <v>45931</v>
       </c>
@@ -10630,7 +10626,7 @@
         <v>9.2413636363636392E-2</v>
       </c>
     </row>
-    <row r="252" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A252" s="1">
         <v>45962</v>
       </c>
@@ -10644,7 +10640,7 @@
         <v>9.2305555555555571E-2</v>
       </c>
     </row>
-    <row r="253" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A253" s="1">
         <v>45992</v>
       </c>

</xml_diff>

<commit_message>
:construction: WTI to understand misleading results
I include the Analysis of Colcap and WTI. The main result is that it seems that WTI is highly correlated with Colcap during the sample period, that could explain the changes.
</commit_message>
<xml_diff>
--- a/R/Input/DATAc.xlsx
+++ b/R/Input/DATAc.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Disco C\Repositorios Git\Monetary-Policy-Shocks-and-Central-bank-information-in-Colombia\R\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{61A7BA06-15EE-486E-B896-9040FC5EED2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E261624B-1EA4-406E-877D-E4527EBB6D47}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16924CE1-2105-4850-9E3D-C08456AD022C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{5935AB3E-80CE-4E87-9EB4-B18D2E64BDED}"/>
   </bookViews>
@@ -54,18 +54,6 @@
     <t>ShockOISL</t>
   </si>
   <si>
-    <t>MP_bloomberg</t>
-  </si>
-  <si>
-    <t>CBI_bloomberg</t>
-  </si>
-  <si>
-    <t>MP_OIS</t>
-  </si>
-  <si>
-    <t>CBI_OIS</t>
-  </si>
-  <si>
     <t>MP_bloo_BEI</t>
   </si>
   <si>
@@ -76,6 +64,18 @@
   </si>
   <si>
     <t>CBI_OIS_BEI</t>
+  </si>
+  <si>
+    <t>MP_OIS_colcap</t>
+  </si>
+  <si>
+    <t>CBI_OIS_colcap</t>
+  </si>
+  <si>
+    <t>MP_bloo_colcap</t>
+  </si>
+  <si>
+    <t>CBI_bloo_colcap</t>
   </si>
 </sst>
 </file>
@@ -478,28 +478,28 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L1" t="s">
+        <v>7</v>
+      </c>
+      <c r="M1" t="s">
         <v>8</v>
       </c>
-      <c r="H1" t="s">
+      <c r="N1" t="s">
         <v>9</v>
-      </c>
-      <c r="I1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>